<commit_message>
AML (マウスレイヤー) を Ctrl / Shift / Win / Alt で解除する (#9)
ryo-aoki-pc/zmk-config-LisM#22 と同じ内容 (LisM 基準)。

- excluded-positions を D / K (&mo SCRL、27 / 34) だけにする。修飾キーの位置
  (A / - / Z / / / Win / Alt) を押すと AML が切れる
- MOUSE_MOVE の修飾キーの位置を &trans にする (BASE と同じ &mt / &kp。タップで文字、
  長押しで修飾キー)
- MOUSE_SCROLL の修飾キーはそのまま。修飾キーとクリック・ホイールを組み合わせるときは
  D / K を押してから修飾キーを押す (例: D → Z → F で Shift + クリック)
- KEYMAP.html / KEYMAP.xlsx を作り直す

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QFG6t92cGtjhGTDoN62Yvg
</commit_message>
<xml_diff>
--- a/KEYMAP.xlsx
+++ b/KEYMAP.xlsx
@@ -6986,7 +6986,7 @@
       <c r="C115" s="7" t="inlineStr">
         <is>
           <t>pos 25
-&amp;kp LCTRL</t>
+&amp;trans</t>
         </is>
       </c>
       <c r="D115" s="7" t="inlineStr">
@@ -7053,7 +7053,7 @@
       <c r="O115" s="7" t="inlineStr">
         <is>
           <t>pos 36
-&amp;kp RCTRL</t>
+&amp;trans</t>
         </is>
       </c>
       <c r="P115" s="7" t="inlineStr">
@@ -7072,7 +7072,7 @@
       <c r="B116" s="9" t="inlineStr"/>
       <c r="C116" s="9" t="inlineStr">
         <is>
-          <t>LCtrl</t>
+          <t>▽</t>
         </is>
       </c>
       <c r="D116" s="9" t="inlineStr"/>
@@ -7096,7 +7096,7 @@
       <c r="N116" s="9" t="inlineStr"/>
       <c r="O116" s="9" t="inlineStr">
         <is>
-          <t>RCtrl</t>
+          <t>▽</t>
         </is>
       </c>
       <c r="P116" s="9" t="inlineStr"/>
@@ -7116,7 +7116,7 @@
       <c r="C117" s="7" t="inlineStr">
         <is>
           <t>pos 39
-&amp;kp LEFT_SHIFT</t>
+&amp;trans</t>
         </is>
       </c>
       <c r="D117" s="7" t="inlineStr">
@@ -7183,7 +7183,7 @@
       <c r="O117" s="7" t="inlineStr">
         <is>
           <t>pos 50
-&amp;kp RIGHT_SHIFT</t>
+&amp;trans</t>
         </is>
       </c>
       <c r="P117" s="7" t="inlineStr">
@@ -7202,7 +7202,7 @@
       <c r="B118" s="9" t="inlineStr"/>
       <c r="C118" s="9" t="inlineStr">
         <is>
-          <t>LShift</t>
+          <t>▽</t>
         </is>
       </c>
       <c r="D118" s="9" t="inlineStr"/>
@@ -7218,7 +7218,7 @@
       <c r="N118" s="9" t="inlineStr"/>
       <c r="O118" s="9" t="inlineStr">
         <is>
-          <t>RShift</t>
+          <t>▽</t>
         </is>
       </c>
       <c r="P118" s="9" t="inlineStr"/>
@@ -7244,13 +7244,13 @@
       <c r="D119" s="7" t="inlineStr">
         <is>
           <t>pos 54
-&amp;kp LEFT_WIN</t>
+&amp;trans</t>
         </is>
       </c>
       <c r="E119" s="7" t="inlineStr">
         <is>
           <t>pos 55
-&amp;kp LEFT_ALT</t>
+&amp;trans</t>
         </is>
       </c>
       <c r="F119" s="7" t="inlineStr">
@@ -7325,12 +7325,12 @@
       <c r="C120" s="9" t="inlineStr"/>
       <c r="D120" s="9" t="inlineStr">
         <is>
-          <t>LWin</t>
+          <t>▽</t>
         </is>
       </c>
       <c r="E120" s="9" t="inlineStr">
         <is>
-          <t>LAlt</t>
+          <t>▽</t>
         </is>
       </c>
       <c r="F120" s="9" t="inlineStr"/>
@@ -14496,7 +14496,7 @@
       <c r="C115" s="7" t="inlineStr">
         <is>
           <t>pos 25
-&amp;kp LCTRL</t>
+&amp;trans</t>
         </is>
       </c>
       <c r="D115" s="7" t="inlineStr">
@@ -14563,7 +14563,7 @@
       <c r="O115" s="7" t="inlineStr">
         <is>
           <t>pos 36
-&amp;kp RCTRL</t>
+&amp;trans</t>
         </is>
       </c>
       <c r="P115" s="7" t="inlineStr">
@@ -14582,7 +14582,7 @@
       <c r="B116" s="9" t="inlineStr"/>
       <c r="C116" s="9" t="inlineStr">
         <is>
-          <t>&amp;kp LCTRL</t>
+          <t>▽</t>
         </is>
       </c>
       <c r="D116" s="9" t="inlineStr"/>
@@ -14606,7 +14606,7 @@
       <c r="N116" s="9" t="inlineStr"/>
       <c r="O116" s="9" t="inlineStr">
         <is>
-          <t>&amp;kp RCTRL</t>
+          <t>▽</t>
         </is>
       </c>
       <c r="P116" s="9" t="inlineStr"/>
@@ -14626,7 +14626,7 @@
       <c r="C117" s="7" t="inlineStr">
         <is>
           <t>pos 39
-&amp;kp LEFT_SHIFT</t>
+&amp;trans</t>
         </is>
       </c>
       <c r="D117" s="7" t="inlineStr">
@@ -14693,7 +14693,7 @@
       <c r="O117" s="7" t="inlineStr">
         <is>
           <t>pos 50
-&amp;kp RIGHT_SHIFT</t>
+&amp;trans</t>
         </is>
       </c>
       <c r="P117" s="7" t="inlineStr">
@@ -14712,7 +14712,7 @@
       <c r="B118" s="9" t="inlineStr"/>
       <c r="C118" s="9" t="inlineStr">
         <is>
-          <t>&amp;kp LEFT_SHIFT</t>
+          <t>▽</t>
         </is>
       </c>
       <c r="D118" s="9" t="inlineStr"/>
@@ -14728,7 +14728,7 @@
       <c r="N118" s="9" t="inlineStr"/>
       <c r="O118" s="9" t="inlineStr">
         <is>
-          <t>&amp;kp RIGHT_SHIFT</t>
+          <t>▽</t>
         </is>
       </c>
       <c r="P118" s="9" t="inlineStr"/>
@@ -14754,13 +14754,13 @@
       <c r="D119" s="7" t="inlineStr">
         <is>
           <t>pos 54
-&amp;kp LEFT_WIN</t>
+&amp;trans</t>
         </is>
       </c>
       <c r="E119" s="7" t="inlineStr">
         <is>
           <t>pos 55
-&amp;kp LEFT_ALT</t>
+&amp;trans</t>
         </is>
       </c>
       <c r="F119" s="7" t="inlineStr">
@@ -14835,12 +14835,12 @@
       <c r="C120" s="9" t="inlineStr"/>
       <c r="D120" s="9" t="inlineStr">
         <is>
-          <t>&amp;kp LEFT_WIN</t>
+          <t>▽</t>
         </is>
       </c>
       <c r="E120" s="9" t="inlineStr">
         <is>
-          <t>&amp;kp LEFT_ALT</t>
+          <t>▽</t>
         </is>
       </c>
       <c r="F120" s="9" t="inlineStr"/>

</xml_diff>